<commit_message>
Update indicator and market explanation logic with documentation and data exports.
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/exports/Explicacoes_Mercado_Bridge_EBITDA.xlsx
+++ b/exports/Explicacoes_Mercado_Bridge_EBITDA.xlsx
@@ -590,7 +590,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B2" t="str">
-        <v>JAN26</v>
+        <v>202601</v>
       </c>
       <c r="C2" t="str">
         <v>Iron Ores</v>
@@ -610,7 +610,7 @@
         <v>MRF7</v>
       </c>
       <c r="B3" t="str">
-        <v>JAN26</v>
+        <v>202601</v>
       </c>
       <c r="C3" t="str">
         <v>Iron Ores</v>
@@ -630,7 +630,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B4" t="str">
-        <v>FEB26</v>
+        <v>202602</v>
       </c>
       <c r="C4" t="str">
         <v>Iron Ores</v>
@@ -650,7 +650,7 @@
         <v>MRF7</v>
       </c>
       <c r="B5" t="str">
-        <v>FEB26</v>
+        <v>202602</v>
       </c>
       <c r="C5" t="str">
         <v>Iron Ores</v>
@@ -670,7 +670,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B6" t="str">
-        <v>MAR26</v>
+        <v>202603</v>
       </c>
       <c r="C6" t="str">
         <v>Iron Ores</v>
@@ -690,7 +690,7 @@
         <v>MRF7</v>
       </c>
       <c r="B7" t="str">
-        <v>MAR26</v>
+        <v>202603</v>
       </c>
       <c r="C7" t="str">
         <v>Iron Ores</v>
@@ -710,7 +710,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B8" t="str">
-        <v>APR26</v>
+        <v>202604</v>
       </c>
       <c r="C8" t="str">
         <v>Iron Ores</v>
@@ -730,7 +730,7 @@
         <v>MRF7</v>
       </c>
       <c r="B9" t="str">
-        <v>APR26</v>
+        <v>202604</v>
       </c>
       <c r="C9" t="str">
         <v>Iron Ores</v>
@@ -750,7 +750,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B10" t="str">
-        <v>MAY26</v>
+        <v>202605</v>
       </c>
       <c r="C10" t="str">
         <v>Iron Ores</v>
@@ -770,7 +770,7 @@
         <v>MRF7</v>
       </c>
       <c r="B11" t="str">
-        <v>MAY26</v>
+        <v>202605</v>
       </c>
       <c r="C11" t="str">
         <v>Iron Ores</v>
@@ -790,7 +790,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B12" t="str">
-        <v>JUN26</v>
+        <v>202606</v>
       </c>
       <c r="C12" t="str">
         <v>Iron Ores</v>
@@ -810,7 +810,7 @@
         <v>MRF7</v>
       </c>
       <c r="B13" t="str">
-        <v>JUN26</v>
+        <v>202606</v>
       </c>
       <c r="C13" t="str">
         <v>Iron Ores</v>
@@ -830,7 +830,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B14" t="str">
-        <v>JUL26</v>
+        <v>202607</v>
       </c>
       <c r="C14" t="str">
         <v>Iron Ores</v>
@@ -850,7 +850,7 @@
         <v>MRF7</v>
       </c>
       <c r="B15" t="str">
-        <v>JUL26</v>
+        <v>202607</v>
       </c>
       <c r="C15" t="str">
         <v>Iron Ores</v>
@@ -870,7 +870,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B16" t="str">
-        <v>AUG26</v>
+        <v>202608</v>
       </c>
       <c r="C16" t="str">
         <v>Iron Ores</v>
@@ -890,7 +890,7 @@
         <v>MRF7</v>
       </c>
       <c r="B17" t="str">
-        <v>AUG26</v>
+        <v>202608</v>
       </c>
       <c r="C17" t="str">
         <v>Iron Ores</v>
@@ -910,7 +910,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B18" t="str">
-        <v>SEP26</v>
+        <v>202609</v>
       </c>
       <c r="C18" t="str">
         <v>Iron Ores</v>
@@ -930,7 +930,7 @@
         <v>MRF7</v>
       </c>
       <c r="B19" t="str">
-        <v>SEP26</v>
+        <v>202609</v>
       </c>
       <c r="C19" t="str">
         <v>Iron Ores</v>
@@ -950,7 +950,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B20" t="str">
-        <v>OCT26</v>
+        <v>202610</v>
       </c>
       <c r="C20" t="str">
         <v>Iron Ores</v>
@@ -970,7 +970,7 @@
         <v>MRF7</v>
       </c>
       <c r="B21" t="str">
-        <v>OCT26</v>
+        <v>202610</v>
       </c>
       <c r="C21" t="str">
         <v>Iron Ores</v>
@@ -990,7 +990,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B22" t="str">
-        <v>NOV26</v>
+        <v>202611</v>
       </c>
       <c r="C22" t="str">
         <v>Iron Ores</v>
@@ -1010,7 +1010,7 @@
         <v>MRF7</v>
       </c>
       <c r="B23" t="str">
-        <v>NOV26</v>
+        <v>202611</v>
       </c>
       <c r="C23" t="str">
         <v>Iron Ores</v>
@@ -1030,7 +1030,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B24" t="str">
-        <v>DEC26</v>
+        <v>202612</v>
       </c>
       <c r="C24" t="str">
         <v>Iron Ores</v>
@@ -1050,7 +1050,7 @@
         <v>MRF7</v>
       </c>
       <c r="B25" t="str">
-        <v>DEC26</v>
+        <v>202612</v>
       </c>
       <c r="C25" t="str">
         <v>Iron Ores</v>
@@ -1070,7 +1070,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B26" t="str">
-        <v>JAN26</v>
+        <v>202601</v>
       </c>
       <c r="C26" t="str">
         <v>Iron Ores</v>
@@ -1090,7 +1090,7 @@
         <v>MRF7</v>
       </c>
       <c r="B27" t="str">
-        <v>JAN26</v>
+        <v>202601</v>
       </c>
       <c r="C27" t="str">
         <v>Iron Ores</v>
@@ -1110,7 +1110,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B28" t="str">
-        <v>FEB26</v>
+        <v>202602</v>
       </c>
       <c r="C28" t="str">
         <v>Iron Ores</v>
@@ -1130,7 +1130,7 @@
         <v>MRF7</v>
       </c>
       <c r="B29" t="str">
-        <v>FEB26</v>
+        <v>202602</v>
       </c>
       <c r="C29" t="str">
         <v>Iron Ores</v>
@@ -1150,7 +1150,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B30" t="str">
-        <v>MAR26</v>
+        <v>202603</v>
       </c>
       <c r="C30" t="str">
         <v>Iron Ores</v>
@@ -1170,7 +1170,7 @@
         <v>MRF7</v>
       </c>
       <c r="B31" t="str">
-        <v>MAR26</v>
+        <v>202603</v>
       </c>
       <c r="C31" t="str">
         <v>Iron Ores</v>
@@ -1190,7 +1190,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B32" t="str">
-        <v>APR26</v>
+        <v>202604</v>
       </c>
       <c r="C32" t="str">
         <v>Iron Ores</v>
@@ -1210,7 +1210,7 @@
         <v>MRF7</v>
       </c>
       <c r="B33" t="str">
-        <v>APR26</v>
+        <v>202604</v>
       </c>
       <c r="C33" t="str">
         <v>Iron Ores</v>
@@ -1230,7 +1230,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B34" t="str">
-        <v>MAY26</v>
+        <v>202605</v>
       </c>
       <c r="C34" t="str">
         <v>Iron Ores</v>
@@ -1250,7 +1250,7 @@
         <v>MRF7</v>
       </c>
       <c r="B35" t="str">
-        <v>MAY26</v>
+        <v>202605</v>
       </c>
       <c r="C35" t="str">
         <v>Iron Ores</v>
@@ -1270,7 +1270,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B36" t="str">
-        <v>JUN26</v>
+        <v>202606</v>
       </c>
       <c r="C36" t="str">
         <v>Iron Ores</v>
@@ -1290,7 +1290,7 @@
         <v>MRF7</v>
       </c>
       <c r="B37" t="str">
-        <v>JUN26</v>
+        <v>202606</v>
       </c>
       <c r="C37" t="str">
         <v>Iron Ores</v>
@@ -1310,7 +1310,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B38" t="str">
-        <v>JUL26</v>
+        <v>202607</v>
       </c>
       <c r="C38" t="str">
         <v>Iron Ores</v>
@@ -1330,7 +1330,7 @@
         <v>MRF7</v>
       </c>
       <c r="B39" t="str">
-        <v>JUL26</v>
+        <v>202607</v>
       </c>
       <c r="C39" t="str">
         <v>Iron Ores</v>
@@ -1350,7 +1350,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B40" t="str">
-        <v>AUG26</v>
+        <v>202608</v>
       </c>
       <c r="C40" t="str">
         <v>Iron Ores</v>
@@ -1370,7 +1370,7 @@
         <v>MRF7</v>
       </c>
       <c r="B41" t="str">
-        <v>AUG26</v>
+        <v>202608</v>
       </c>
       <c r="C41" t="str">
         <v>Iron Ores</v>
@@ -1390,7 +1390,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B42" t="str">
-        <v>SEP26</v>
+        <v>202609</v>
       </c>
       <c r="C42" t="str">
         <v>Iron Ores</v>
@@ -1410,7 +1410,7 @@
         <v>MRF7</v>
       </c>
       <c r="B43" t="str">
-        <v>SEP26</v>
+        <v>202609</v>
       </c>
       <c r="C43" t="str">
         <v>Iron Ores</v>
@@ -1430,7 +1430,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B44" t="str">
-        <v>OCT26</v>
+        <v>202610</v>
       </c>
       <c r="C44" t="str">
         <v>Iron Ores</v>
@@ -1450,7 +1450,7 @@
         <v>MRF7</v>
       </c>
       <c r="B45" t="str">
-        <v>OCT26</v>
+        <v>202610</v>
       </c>
       <c r="C45" t="str">
         <v>Iron Ores</v>
@@ -1470,7 +1470,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B46" t="str">
-        <v>NOV26</v>
+        <v>202611</v>
       </c>
       <c r="C46" t="str">
         <v>Iron Ores</v>
@@ -1490,7 +1490,7 @@
         <v>MRF7</v>
       </c>
       <c r="B47" t="str">
-        <v>NOV26</v>
+        <v>202611</v>
       </c>
       <c r="C47" t="str">
         <v>Iron Ores</v>
@@ -1510,7 +1510,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B48" t="str">
-        <v>DEC26</v>
+        <v>202612</v>
       </c>
       <c r="C48" t="str">
         <v>Iron Ores</v>
@@ -1530,7 +1530,7 @@
         <v>MRF7</v>
       </c>
       <c r="B49" t="str">
-        <v>DEC26</v>
+        <v>202612</v>
       </c>
       <c r="C49" t="str">
         <v>Iron Ores</v>
@@ -1550,7 +1550,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B50" t="str">
-        <v>JAN26</v>
+        <v>202601</v>
       </c>
       <c r="C50" t="str">
         <v>Iron Ores</v>
@@ -1570,7 +1570,7 @@
         <v>MRF7</v>
       </c>
       <c r="B51" t="str">
-        <v>JAN26</v>
+        <v>202601</v>
       </c>
       <c r="C51" t="str">
         <v>Iron Ores</v>
@@ -1590,7 +1590,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B52" t="str">
-        <v>FEB26</v>
+        <v>202602</v>
       </c>
       <c r="C52" t="str">
         <v>Iron Ores</v>
@@ -1610,7 +1610,7 @@
         <v>MRF7</v>
       </c>
       <c r="B53" t="str">
-        <v>FEB26</v>
+        <v>202602</v>
       </c>
       <c r="C53" t="str">
         <v>Iron Ores</v>
@@ -1630,7 +1630,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B54" t="str">
-        <v>MAR26</v>
+        <v>202603</v>
       </c>
       <c r="C54" t="str">
         <v>Iron Ores</v>
@@ -1650,7 +1650,7 @@
         <v>MRF7</v>
       </c>
       <c r="B55" t="str">
-        <v>MAR26</v>
+        <v>202603</v>
       </c>
       <c r="C55" t="str">
         <v>Iron Ores</v>
@@ -1670,7 +1670,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B56" t="str">
-        <v>APR26</v>
+        <v>202604</v>
       </c>
       <c r="C56" t="str">
         <v>Iron Ores</v>
@@ -1690,7 +1690,7 @@
         <v>MRF7</v>
       </c>
       <c r="B57" t="str">
-        <v>APR26</v>
+        <v>202604</v>
       </c>
       <c r="C57" t="str">
         <v>Iron Ores</v>
@@ -1710,7 +1710,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B58" t="str">
-        <v>MAY26</v>
+        <v>202605</v>
       </c>
       <c r="C58" t="str">
         <v>Iron Ores</v>
@@ -1730,7 +1730,7 @@
         <v>MRF7</v>
       </c>
       <c r="B59" t="str">
-        <v>MAY26</v>
+        <v>202605</v>
       </c>
       <c r="C59" t="str">
         <v>Iron Ores</v>
@@ -1750,7 +1750,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B60" t="str">
-        <v>JUN26</v>
+        <v>202606</v>
       </c>
       <c r="C60" t="str">
         <v>Iron Ores</v>
@@ -1770,7 +1770,7 @@
         <v>MRF7</v>
       </c>
       <c r="B61" t="str">
-        <v>JUN26</v>
+        <v>202606</v>
       </c>
       <c r="C61" t="str">
         <v>Iron Ores</v>
@@ -1790,7 +1790,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B62" t="str">
-        <v>JUL26</v>
+        <v>202607</v>
       </c>
       <c r="C62" t="str">
         <v>Iron Ores</v>
@@ -1810,7 +1810,7 @@
         <v>MRF7</v>
       </c>
       <c r="B63" t="str">
-        <v>JUL26</v>
+        <v>202607</v>
       </c>
       <c r="C63" t="str">
         <v>Iron Ores</v>
@@ -1830,7 +1830,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B64" t="str">
-        <v>AUG26</v>
+        <v>202608</v>
       </c>
       <c r="C64" t="str">
         <v>Iron Ores</v>
@@ -1850,7 +1850,7 @@
         <v>MRF7</v>
       </c>
       <c r="B65" t="str">
-        <v>AUG26</v>
+        <v>202608</v>
       </c>
       <c r="C65" t="str">
         <v>Iron Ores</v>
@@ -1870,7 +1870,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B66" t="str">
-        <v>SEP26</v>
+        <v>202609</v>
       </c>
       <c r="C66" t="str">
         <v>Iron Ores</v>
@@ -1890,7 +1890,7 @@
         <v>MRF7</v>
       </c>
       <c r="B67" t="str">
-        <v>SEP26</v>
+        <v>202609</v>
       </c>
       <c r="C67" t="str">
         <v>Iron Ores</v>
@@ -1910,7 +1910,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B68" t="str">
-        <v>OCT26</v>
+        <v>202610</v>
       </c>
       <c r="C68" t="str">
         <v>Iron Ores</v>
@@ -1930,7 +1930,7 @@
         <v>MRF7</v>
       </c>
       <c r="B69" t="str">
-        <v>OCT26</v>
+        <v>202610</v>
       </c>
       <c r="C69" t="str">
         <v>Iron Ores</v>
@@ -1950,7 +1950,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B70" t="str">
-        <v>NOV26</v>
+        <v>202611</v>
       </c>
       <c r="C70" t="str">
         <v>Iron Ores</v>
@@ -1970,7 +1970,7 @@
         <v>MRF7</v>
       </c>
       <c r="B71" t="str">
-        <v>NOV26</v>
+        <v>202611</v>
       </c>
       <c r="C71" t="str">
         <v>Iron Ores</v>
@@ -1990,7 +1990,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B72" t="str">
-        <v>DEC26</v>
+        <v>202612</v>
       </c>
       <c r="C72" t="str">
         <v>Iron Ores</v>
@@ -2010,7 +2010,7 @@
         <v>MRF7</v>
       </c>
       <c r="B73" t="str">
-        <v>DEC26</v>
+        <v>202612</v>
       </c>
       <c r="C73" t="str">
         <v>Iron Ores</v>
@@ -2030,7 +2030,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B74" t="str">
-        <v>JAN26</v>
+        <v>202601</v>
       </c>
       <c r="C74" t="str">
         <v>Iron Ores</v>
@@ -2050,7 +2050,7 @@
         <v>MRF7</v>
       </c>
       <c r="B75" t="str">
-        <v>JAN26</v>
+        <v>202601</v>
       </c>
       <c r="C75" t="str">
         <v>Iron Ores</v>
@@ -2070,7 +2070,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B76" t="str">
-        <v>FEB26</v>
+        <v>202602</v>
       </c>
       <c r="C76" t="str">
         <v>Iron Ores</v>
@@ -2090,7 +2090,7 @@
         <v>MRF7</v>
       </c>
       <c r="B77" t="str">
-        <v>FEB26</v>
+        <v>202602</v>
       </c>
       <c r="C77" t="str">
         <v>Iron Ores</v>
@@ -2110,7 +2110,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B78" t="str">
-        <v>MAR26</v>
+        <v>202603</v>
       </c>
       <c r="C78" t="str">
         <v>Iron Ores</v>
@@ -2130,7 +2130,7 @@
         <v>MRF7</v>
       </c>
       <c r="B79" t="str">
-        <v>MAR26</v>
+        <v>202603</v>
       </c>
       <c r="C79" t="str">
         <v>Iron Ores</v>
@@ -2150,7 +2150,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B80" t="str">
-        <v>APR26</v>
+        <v>202604</v>
       </c>
       <c r="C80" t="str">
         <v>Iron Ores</v>
@@ -2170,7 +2170,7 @@
         <v>MRF7</v>
       </c>
       <c r="B81" t="str">
-        <v>APR26</v>
+        <v>202604</v>
       </c>
       <c r="C81" t="str">
         <v>Iron Ores</v>
@@ -2190,7 +2190,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B82" t="str">
-        <v>MAY26</v>
+        <v>202605</v>
       </c>
       <c r="C82" t="str">
         <v>Iron Ores</v>
@@ -2210,7 +2210,7 @@
         <v>MRF7</v>
       </c>
       <c r="B83" t="str">
-        <v>MAY26</v>
+        <v>202605</v>
       </c>
       <c r="C83" t="str">
         <v>Iron Ores</v>
@@ -2230,7 +2230,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B84" t="str">
-        <v>JUN26</v>
+        <v>202606</v>
       </c>
       <c r="C84" t="str">
         <v>Iron Ores</v>
@@ -2250,7 +2250,7 @@
         <v>MRF7</v>
       </c>
       <c r="B85" t="str">
-        <v>JUN26</v>
+        <v>202606</v>
       </c>
       <c r="C85" t="str">
         <v>Iron Ores</v>
@@ -2270,7 +2270,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B86" t="str">
-        <v>JUL26</v>
+        <v>202607</v>
       </c>
       <c r="C86" t="str">
         <v>Iron Ores</v>
@@ -2290,7 +2290,7 @@
         <v>MRF7</v>
       </c>
       <c r="B87" t="str">
-        <v>JUL26</v>
+        <v>202607</v>
       </c>
       <c r="C87" t="str">
         <v>Iron Ores</v>
@@ -2310,7 +2310,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B88" t="str">
-        <v>AUG26</v>
+        <v>202608</v>
       </c>
       <c r="C88" t="str">
         <v>Iron Ores</v>
@@ -2330,7 +2330,7 @@
         <v>MRF7</v>
       </c>
       <c r="B89" t="str">
-        <v>AUG26</v>
+        <v>202608</v>
       </c>
       <c r="C89" t="str">
         <v>Iron Ores</v>
@@ -2350,7 +2350,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B90" t="str">
-        <v>SEP26</v>
+        <v>202609</v>
       </c>
       <c r="C90" t="str">
         <v>Iron Ores</v>
@@ -2370,7 +2370,7 @@
         <v>MRF7</v>
       </c>
       <c r="B91" t="str">
-        <v>SEP26</v>
+        <v>202609</v>
       </c>
       <c r="C91" t="str">
         <v>Iron Ores</v>
@@ -2390,7 +2390,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B92" t="str">
-        <v>OCT26</v>
+        <v>202610</v>
       </c>
       <c r="C92" t="str">
         <v>Iron Ores</v>
@@ -2410,7 +2410,7 @@
         <v>MRF7</v>
       </c>
       <c r="B93" t="str">
-        <v>OCT26</v>
+        <v>202610</v>
       </c>
       <c r="C93" t="str">
         <v>Iron Ores</v>
@@ -2430,7 +2430,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B94" t="str">
-        <v>NOV26</v>
+        <v>202611</v>
       </c>
       <c r="C94" t="str">
         <v>Iron Ores</v>
@@ -2450,7 +2450,7 @@
         <v>MRF7</v>
       </c>
       <c r="B95" t="str">
-        <v>NOV26</v>
+        <v>202611</v>
       </c>
       <c r="C95" t="str">
         <v>Iron Ores</v>
@@ -2470,7 +2470,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B96" t="str">
-        <v>DEC26</v>
+        <v>202612</v>
       </c>
       <c r="C96" t="str">
         <v>Iron Ores</v>
@@ -2490,7 +2490,7 @@
         <v>MRF7</v>
       </c>
       <c r="B97" t="str">
-        <v>DEC26</v>
+        <v>202612</v>
       </c>
       <c r="C97" t="str">
         <v>Iron Ores</v>
@@ -2510,7 +2510,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B98" t="str">
-        <v>JAN26</v>
+        <v>202601</v>
       </c>
       <c r="C98" t="str">
         <v>Iron Ores</v>
@@ -2530,7 +2530,7 @@
         <v>MRF7</v>
       </c>
       <c r="B99" t="str">
-        <v>JAN26</v>
+        <v>202601</v>
       </c>
       <c r="C99" t="str">
         <v>Iron Ores</v>
@@ -2550,7 +2550,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B100" t="str">
-        <v>FEB26</v>
+        <v>202602</v>
       </c>
       <c r="C100" t="str">
         <v>Iron Ores</v>
@@ -2570,7 +2570,7 @@
         <v>MRF7</v>
       </c>
       <c r="B101" t="str">
-        <v>FEB26</v>
+        <v>202602</v>
       </c>
       <c r="C101" t="str">
         <v>Iron Ores</v>
@@ -2590,7 +2590,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B102" t="str">
-        <v>MAR26</v>
+        <v>202603</v>
       </c>
       <c r="C102" t="str">
         <v>Iron Ores</v>
@@ -2610,7 +2610,7 @@
         <v>MRF7</v>
       </c>
       <c r="B103" t="str">
-        <v>MAR26</v>
+        <v>202603</v>
       </c>
       <c r="C103" t="str">
         <v>Iron Ores</v>
@@ -2630,7 +2630,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B104" t="str">
-        <v>APR26</v>
+        <v>202604</v>
       </c>
       <c r="C104" t="str">
         <v>Iron Ores</v>
@@ -2650,7 +2650,7 @@
         <v>MRF7</v>
       </c>
       <c r="B105" t="str">
-        <v>APR26</v>
+        <v>202604</v>
       </c>
       <c r="C105" t="str">
         <v>Iron Ores</v>
@@ -2670,7 +2670,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B106" t="str">
-        <v>MAY26</v>
+        <v>202605</v>
       </c>
       <c r="C106" t="str">
         <v>Iron Ores</v>
@@ -2690,7 +2690,7 @@
         <v>MRF7</v>
       </c>
       <c r="B107" t="str">
-        <v>MAY26</v>
+        <v>202605</v>
       </c>
       <c r="C107" t="str">
         <v>Iron Ores</v>
@@ -2710,7 +2710,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B108" t="str">
-        <v>JUN26</v>
+        <v>202606</v>
       </c>
       <c r="C108" t="str">
         <v>Iron Ores</v>
@@ -2730,7 +2730,7 @@
         <v>MRF7</v>
       </c>
       <c r="B109" t="str">
-        <v>JUN26</v>
+        <v>202606</v>
       </c>
       <c r="C109" t="str">
         <v>Iron Ores</v>
@@ -2750,7 +2750,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B110" t="str">
-        <v>JUL26</v>
+        <v>202607</v>
       </c>
       <c r="C110" t="str">
         <v>Iron Ores</v>
@@ -2770,7 +2770,7 @@
         <v>MRF7</v>
       </c>
       <c r="B111" t="str">
-        <v>JUL26</v>
+        <v>202607</v>
       </c>
       <c r="C111" t="str">
         <v>Iron Ores</v>
@@ -2790,7 +2790,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B112" t="str">
-        <v>AUG26</v>
+        <v>202608</v>
       </c>
       <c r="C112" t="str">
         <v>Iron Ores</v>
@@ -2810,7 +2810,7 @@
         <v>MRF7</v>
       </c>
       <c r="B113" t="str">
-        <v>AUG26</v>
+        <v>202608</v>
       </c>
       <c r="C113" t="str">
         <v>Iron Ores</v>
@@ -2830,7 +2830,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B114" t="str">
-        <v>SEP26</v>
+        <v>202609</v>
       </c>
       <c r="C114" t="str">
         <v>Iron Ores</v>
@@ -2850,7 +2850,7 @@
         <v>MRF7</v>
       </c>
       <c r="B115" t="str">
-        <v>SEP26</v>
+        <v>202609</v>
       </c>
       <c r="C115" t="str">
         <v>Iron Ores</v>
@@ -2870,7 +2870,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B116" t="str">
-        <v>OCT26</v>
+        <v>202610</v>
       </c>
       <c r="C116" t="str">
         <v>Iron Ores</v>
@@ -2890,7 +2890,7 @@
         <v>MRF7</v>
       </c>
       <c r="B117" t="str">
-        <v>OCT26</v>
+        <v>202610</v>
       </c>
       <c r="C117" t="str">
         <v>Iron Ores</v>
@@ -2910,7 +2910,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B118" t="str">
-        <v>NOV26</v>
+        <v>202611</v>
       </c>
       <c r="C118" t="str">
         <v>Iron Ores</v>
@@ -2930,7 +2930,7 @@
         <v>MRF7</v>
       </c>
       <c r="B119" t="str">
-        <v>NOV26</v>
+        <v>202611</v>
       </c>
       <c r="C119" t="str">
         <v>Iron Ores</v>
@@ -2950,7 +2950,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B120" t="str">
-        <v>DEC26</v>
+        <v>202612</v>
       </c>
       <c r="C120" t="str">
         <v>Iron Ores</v>
@@ -2970,7 +2970,7 @@
         <v>MRF7</v>
       </c>
       <c r="B121" t="str">
-        <v>DEC26</v>
+        <v>202612</v>
       </c>
       <c r="C121" t="str">
         <v>Iron Ores</v>
@@ -2990,7 +2990,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B122" t="str">
-        <v>JAN26</v>
+        <v>202601</v>
       </c>
       <c r="C122" t="str">
         <v>Iron Ores</v>
@@ -3010,7 +3010,7 @@
         <v>MRF7</v>
       </c>
       <c r="B123" t="str">
-        <v>JAN26</v>
+        <v>202601</v>
       </c>
       <c r="C123" t="str">
         <v>Iron Ores</v>
@@ -3030,7 +3030,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B124" t="str">
-        <v>FEB26</v>
+        <v>202602</v>
       </c>
       <c r="C124" t="str">
         <v>Iron Ores</v>
@@ -3050,7 +3050,7 @@
         <v>MRF7</v>
       </c>
       <c r="B125" t="str">
-        <v>FEB26</v>
+        <v>202602</v>
       </c>
       <c r="C125" t="str">
         <v>Iron Ores</v>
@@ -3070,7 +3070,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B126" t="str">
-        <v>MAR26</v>
+        <v>202603</v>
       </c>
       <c r="C126" t="str">
         <v>Iron Ores</v>
@@ -3090,7 +3090,7 @@
         <v>MRF7</v>
       </c>
       <c r="B127" t="str">
-        <v>MAR26</v>
+        <v>202603</v>
       </c>
       <c r="C127" t="str">
         <v>Iron Ores</v>
@@ -3110,7 +3110,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B128" t="str">
-        <v>APR26</v>
+        <v>202604</v>
       </c>
       <c r="C128" t="str">
         <v>Iron Ores</v>
@@ -3130,7 +3130,7 @@
         <v>MRF7</v>
       </c>
       <c r="B129" t="str">
-        <v>APR26</v>
+        <v>202604</v>
       </c>
       <c r="C129" t="str">
         <v>Iron Ores</v>
@@ -3150,7 +3150,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B130" t="str">
-        <v>MAY26</v>
+        <v>202605</v>
       </c>
       <c r="C130" t="str">
         <v>Iron Ores</v>
@@ -3170,7 +3170,7 @@
         <v>MRF7</v>
       </c>
       <c r="B131" t="str">
-        <v>MAY26</v>
+        <v>202605</v>
       </c>
       <c r="C131" t="str">
         <v>Iron Ores</v>
@@ -3190,7 +3190,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B132" t="str">
-        <v>JUN26</v>
+        <v>202606</v>
       </c>
       <c r="C132" t="str">
         <v>Iron Ores</v>
@@ -3210,7 +3210,7 @@
         <v>MRF7</v>
       </c>
       <c r="B133" t="str">
-        <v>JUN26</v>
+        <v>202606</v>
       </c>
       <c r="C133" t="str">
         <v>Iron Ores</v>
@@ -3230,7 +3230,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B134" t="str">
-        <v>JUL26</v>
+        <v>202607</v>
       </c>
       <c r="C134" t="str">
         <v>Iron Ores</v>
@@ -3250,7 +3250,7 @@
         <v>MRF7</v>
       </c>
       <c r="B135" t="str">
-        <v>JUL26</v>
+        <v>202607</v>
       </c>
       <c r="C135" t="str">
         <v>Iron Ores</v>
@@ -3270,7 +3270,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B136" t="str">
-        <v>AUG26</v>
+        <v>202608</v>
       </c>
       <c r="C136" t="str">
         <v>Iron Ores</v>
@@ -3290,7 +3290,7 @@
         <v>MRF7</v>
       </c>
       <c r="B137" t="str">
-        <v>AUG26</v>
+        <v>202608</v>
       </c>
       <c r="C137" t="str">
         <v>Iron Ores</v>
@@ -3310,7 +3310,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B138" t="str">
-        <v>SEP26</v>
+        <v>202609</v>
       </c>
       <c r="C138" t="str">
         <v>Iron Ores</v>
@@ -3330,7 +3330,7 @@
         <v>MRF7</v>
       </c>
       <c r="B139" t="str">
-        <v>SEP26</v>
+        <v>202609</v>
       </c>
       <c r="C139" t="str">
         <v>Iron Ores</v>
@@ -3350,7 +3350,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B140" t="str">
-        <v>OCT26</v>
+        <v>202610</v>
       </c>
       <c r="C140" t="str">
         <v>Iron Ores</v>
@@ -3370,7 +3370,7 @@
         <v>MRF7</v>
       </c>
       <c r="B141" t="str">
-        <v>OCT26</v>
+        <v>202610</v>
       </c>
       <c r="C141" t="str">
         <v>Iron Ores</v>
@@ -3390,7 +3390,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B142" t="str">
-        <v>NOV26</v>
+        <v>202611</v>
       </c>
       <c r="C142" t="str">
         <v>Iron Ores</v>
@@ -3410,7 +3410,7 @@
         <v>MRF7</v>
       </c>
       <c r="B143" t="str">
-        <v>NOV26</v>
+        <v>202611</v>
       </c>
       <c r="C143" t="str">
         <v>Iron Ores</v>
@@ -3430,7 +3430,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B144" t="str">
-        <v>DEC26</v>
+        <v>202612</v>
       </c>
       <c r="C144" t="str">
         <v>Iron Ores</v>
@@ -3450,7 +3450,7 @@
         <v>MRF7</v>
       </c>
       <c r="B145" t="str">
-        <v>DEC26</v>
+        <v>202612</v>
       </c>
       <c r="C145" t="str">
         <v>Iron Ores</v>
@@ -3470,7 +3470,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B146" t="str">
-        <v>JAN26</v>
+        <v>202601</v>
       </c>
       <c r="C146" t="str">
         <v>Iron Ores</v>
@@ -3487,7 +3487,7 @@
         <v>MRF7</v>
       </c>
       <c r="B147" t="str">
-        <v>JAN26</v>
+        <v>202601</v>
       </c>
       <c r="C147" t="str">
         <v>Iron Ores</v>
@@ -3504,7 +3504,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B148" t="str">
-        <v>FEB26</v>
+        <v>202602</v>
       </c>
       <c r="C148" t="str">
         <v>Iron Ores</v>
@@ -3521,7 +3521,7 @@
         <v>MRF7</v>
       </c>
       <c r="B149" t="str">
-        <v>FEB26</v>
+        <v>202602</v>
       </c>
       <c r="C149" t="str">
         <v>Iron Ores</v>
@@ -3538,7 +3538,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B150" t="str">
-        <v>MAR26</v>
+        <v>202603</v>
       </c>
       <c r="C150" t="str">
         <v>Iron Ores</v>
@@ -3555,7 +3555,7 @@
         <v>MRF7</v>
       </c>
       <c r="B151" t="str">
-        <v>MAR26</v>
+        <v>202603</v>
       </c>
       <c r="C151" t="str">
         <v>Iron Ores</v>
@@ -3572,7 +3572,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B152" t="str">
-        <v>APR26</v>
+        <v>202604</v>
       </c>
       <c r="C152" t="str">
         <v>Iron Ores</v>
@@ -3589,7 +3589,7 @@
         <v>MRF7</v>
       </c>
       <c r="B153" t="str">
-        <v>APR26</v>
+        <v>202604</v>
       </c>
       <c r="C153" t="str">
         <v>Iron Ores</v>
@@ -3606,7 +3606,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B154" t="str">
-        <v>MAY26</v>
+        <v>202605</v>
       </c>
       <c r="C154" t="str">
         <v>Iron Ores</v>
@@ -3623,7 +3623,7 @@
         <v>MRF7</v>
       </c>
       <c r="B155" t="str">
-        <v>MAY26</v>
+        <v>202605</v>
       </c>
       <c r="C155" t="str">
         <v>Iron Ores</v>
@@ -3640,7 +3640,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B156" t="str">
-        <v>JUN26</v>
+        <v>202606</v>
       </c>
       <c r="C156" t="str">
         <v>Iron Ores</v>
@@ -3657,7 +3657,7 @@
         <v>MRF7</v>
       </c>
       <c r="B157" t="str">
-        <v>JUN26</v>
+        <v>202606</v>
       </c>
       <c r="C157" t="str">
         <v>Iron Ores</v>
@@ -3674,7 +3674,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B158" t="str">
-        <v>JUL26</v>
+        <v>202607</v>
       </c>
       <c r="C158" t="str">
         <v>Iron Ores</v>
@@ -3691,7 +3691,7 @@
         <v>MRF7</v>
       </c>
       <c r="B159" t="str">
-        <v>JUL26</v>
+        <v>202607</v>
       </c>
       <c r="C159" t="str">
         <v>Iron Ores</v>
@@ -3708,7 +3708,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B160" t="str">
-        <v>AUG26</v>
+        <v>202608</v>
       </c>
       <c r="C160" t="str">
         <v>Iron Ores</v>
@@ -3725,7 +3725,7 @@
         <v>MRF7</v>
       </c>
       <c r="B161" t="str">
-        <v>AUG26</v>
+        <v>202608</v>
       </c>
       <c r="C161" t="str">
         <v>Iron Ores</v>
@@ -3742,7 +3742,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B162" t="str">
-        <v>SEP26</v>
+        <v>202609</v>
       </c>
       <c r="C162" t="str">
         <v>Iron Ores</v>
@@ -3759,7 +3759,7 @@
         <v>MRF7</v>
       </c>
       <c r="B163" t="str">
-        <v>SEP26</v>
+        <v>202609</v>
       </c>
       <c r="C163" t="str">
         <v>Iron Ores</v>
@@ -3776,7 +3776,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B164" t="str">
-        <v>OCT26</v>
+        <v>202610</v>
       </c>
       <c r="C164" t="str">
         <v>Iron Ores</v>
@@ -3793,7 +3793,7 @@
         <v>MRF7</v>
       </c>
       <c r="B165" t="str">
-        <v>OCT26</v>
+        <v>202610</v>
       </c>
       <c r="C165" t="str">
         <v>Iron Ores</v>
@@ -3810,7 +3810,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B166" t="str">
-        <v>NOV26</v>
+        <v>202611</v>
       </c>
       <c r="C166" t="str">
         <v>Iron Ores</v>
@@ -3827,7 +3827,7 @@
         <v>MRF7</v>
       </c>
       <c r="B167" t="str">
-        <v>NOV26</v>
+        <v>202611</v>
       </c>
       <c r="C167" t="str">
         <v>Iron Ores</v>
@@ -3844,7 +3844,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B168" t="str">
-        <v>DEC26</v>
+        <v>202612</v>
       </c>
       <c r="C168" t="str">
         <v>Iron Ores</v>
@@ -3861,7 +3861,7 @@
         <v>MRF7</v>
       </c>
       <c r="B169" t="str">
-        <v>DEC26</v>
+        <v>202612</v>
       </c>
       <c r="C169" t="str">
         <v>Iron Ores</v>
@@ -3878,7 +3878,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B170" t="str">
-        <v>JAN26</v>
+        <v>202601</v>
       </c>
       <c r="C170" t="str">
         <v>Iron Ores</v>
@@ -3895,7 +3895,7 @@
         <v>MRF7</v>
       </c>
       <c r="B171" t="str">
-        <v>JAN26</v>
+        <v>202601</v>
       </c>
       <c r="C171" t="str">
         <v>Iron Ores</v>
@@ -3912,7 +3912,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B172" t="str">
-        <v>FEB26</v>
+        <v>202602</v>
       </c>
       <c r="C172" t="str">
         <v>Iron Ores</v>
@@ -3929,7 +3929,7 @@
         <v>MRF7</v>
       </c>
       <c r="B173" t="str">
-        <v>FEB26</v>
+        <v>202602</v>
       </c>
       <c r="C173" t="str">
         <v>Iron Ores</v>
@@ -3946,7 +3946,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B174" t="str">
-        <v>MAR26</v>
+        <v>202603</v>
       </c>
       <c r="C174" t="str">
         <v>Iron Ores</v>
@@ -3963,7 +3963,7 @@
         <v>MRF7</v>
       </c>
       <c r="B175" t="str">
-        <v>MAR26</v>
+        <v>202603</v>
       </c>
       <c r="C175" t="str">
         <v>Iron Ores</v>
@@ -3980,7 +3980,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B176" t="str">
-        <v>APR26</v>
+        <v>202604</v>
       </c>
       <c r="C176" t="str">
         <v>Iron Ores</v>
@@ -3997,7 +3997,7 @@
         <v>MRF7</v>
       </c>
       <c r="B177" t="str">
-        <v>APR26</v>
+        <v>202604</v>
       </c>
       <c r="C177" t="str">
         <v>Iron Ores</v>
@@ -4014,7 +4014,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B178" t="str">
-        <v>MAY26</v>
+        <v>202605</v>
       </c>
       <c r="C178" t="str">
         <v>Iron Ores</v>
@@ -4031,7 +4031,7 @@
         <v>MRF7</v>
       </c>
       <c r="B179" t="str">
-        <v>MAY26</v>
+        <v>202605</v>
       </c>
       <c r="C179" t="str">
         <v>Iron Ores</v>
@@ -4048,7 +4048,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B180" t="str">
-        <v>JUN26</v>
+        <v>202606</v>
       </c>
       <c r="C180" t="str">
         <v>Iron Ores</v>
@@ -4065,7 +4065,7 @@
         <v>MRF7</v>
       </c>
       <c r="B181" t="str">
-        <v>JUN26</v>
+        <v>202606</v>
       </c>
       <c r="C181" t="str">
         <v>Iron Ores</v>
@@ -4082,7 +4082,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B182" t="str">
-        <v>JUL26</v>
+        <v>202607</v>
       </c>
       <c r="C182" t="str">
         <v>Iron Ores</v>
@@ -4099,7 +4099,7 @@
         <v>MRF7</v>
       </c>
       <c r="B183" t="str">
-        <v>JUL26</v>
+        <v>202607</v>
       </c>
       <c r="C183" t="str">
         <v>Iron Ores</v>
@@ -4116,7 +4116,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B184" t="str">
-        <v>AUG26</v>
+        <v>202608</v>
       </c>
       <c r="C184" t="str">
         <v>Iron Ores</v>
@@ -4133,7 +4133,7 @@
         <v>MRF7</v>
       </c>
       <c r="B185" t="str">
-        <v>AUG26</v>
+        <v>202608</v>
       </c>
       <c r="C185" t="str">
         <v>Iron Ores</v>
@@ -4150,7 +4150,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B186" t="str">
-        <v>SEP26</v>
+        <v>202609</v>
       </c>
       <c r="C186" t="str">
         <v>Iron Ores</v>
@@ -4167,7 +4167,7 @@
         <v>MRF7</v>
       </c>
       <c r="B187" t="str">
-        <v>SEP26</v>
+        <v>202609</v>
       </c>
       <c r="C187" t="str">
         <v>Iron Ores</v>
@@ -4184,7 +4184,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B188" t="str">
-        <v>OCT26</v>
+        <v>202610</v>
       </c>
       <c r="C188" t="str">
         <v>Iron Ores</v>
@@ -4201,7 +4201,7 @@
         <v>MRF7</v>
       </c>
       <c r="B189" t="str">
-        <v>OCT26</v>
+        <v>202610</v>
       </c>
       <c r="C189" t="str">
         <v>Iron Ores</v>
@@ -4218,7 +4218,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B190" t="str">
-        <v>NOV26</v>
+        <v>202611</v>
       </c>
       <c r="C190" t="str">
         <v>Iron Ores</v>
@@ -4235,7 +4235,7 @@
         <v>MRF7</v>
       </c>
       <c r="B191" t="str">
-        <v>NOV26</v>
+        <v>202611</v>
       </c>
       <c r="C191" t="str">
         <v>Iron Ores</v>
@@ -4252,7 +4252,7 @@
         <v>BUDGET</v>
       </c>
       <c r="B192" t="str">
-        <v>DEC26</v>
+        <v>202612</v>
       </c>
       <c r="C192" t="str">
         <v>Iron Ores</v>
@@ -4269,7 +4269,7 @@
         <v>MRF7</v>
       </c>
       <c r="B193" t="str">
-        <v>DEC26</v>
+        <v>202612</v>
       </c>
       <c r="C193" t="str">
         <v>Iron Ores</v>

</xml_diff>